<commit_message>
Trying to fix errors
updated to make better
</commit_message>
<xml_diff>
--- a/SubRES_TMPL/SubRES_SUP_H2Curtail.xlsx
+++ b/SubRES_TMPL/SubRES_SUP_H2Curtail.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="94">
   <si>
     <t xml:space="preserve">TIMES-Ireland Model</t>
   </si>
@@ -83,7 +83,7 @@
     <t xml:space="preserve">ELCC (surplus) -&gt; P-CURT -&gt; ELCCUR -&gt; SH2PCELC_CUR -&gt; SUPH2GC. ELCCUR LimType FX = all curtailed electricity MUST be electrolysed (use LO for 'up to all').</t>
   </si>
   <si>
-    <t xml:space="preserve">Use together with Scen_PWR_RES_MustRun (renewables FX) and ELCC LimType = FX in VT_IE_PWR &gt; Commodities &gt; J21. Electrolyser data = placeholders; keep identical to SH2PCELC_01 in SubRES_SUP_Hydrogen.</t>
+    <t xml:space="preserve">Use with Scen_PWR_RES_MustRun (renewables FX from 2025 + bans P-CURT-DUMP from 2025) and ELCC LimType = FX in VT_IE_PWR &gt; Commodities &gt; J21. P-CURT-DUMP lets surplus be discarded in 2018-2024 (before electrolysers exist / historic calibration years).</t>
   </si>
   <si>
     <t xml:space="preserve">~FI_Comm</t>
@@ -210,6 +210,12 @@
   </si>
   <si>
     <t xml:space="preserve">YES</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P-CURT-DUMP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dump of curtailed electricity (allowed before 2025 only)</t>
   </si>
   <si>
     <t xml:space="preserve">~FI_T</t>
@@ -428,35 +434,35 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -715,81 +721,81 @@
   <dimension ref="A16:B32"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="90"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="90"/>
   </cols>
   <sheetData>
-    <row r="16" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="1" t="s">
+    <row r="16" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="2" t="s">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B19" s="3" t="s">
+      <c r="B19" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="2" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B20" s="3" t="s">
+      <c r="B20" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="2" t="s">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B21" s="3" t="s">
+      <c r="B21" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="2" t="s">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B23" s="3" t="s">
+      <c r="B23" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="2" t="s">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B26" s="3" t="s">
+      <c r="B26" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="2" t="s">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B29" s="3" t="s">
+      <c r="B29" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="2" t="s">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B30" s="3" t="s">
+      <c r="B30" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="2" t="s">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B31" s="3" t="s">
+      <c r="B31" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B32" s="0" t="s">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B32" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -812,39 +818,39 @@
   <dimension ref="A1:P24"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="10" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="14" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="10" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="14" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="10"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
         <v>22</v>
       </c>
@@ -870,7 +876,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
         <v>30</v>
       </c>
@@ -892,32 +898,32 @@
       <c r="G7" s="7"/>
       <c r="H7" s="7"/>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="B8" s="0" t="s">
+      <c r="B8" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="C8" s="0" t="s">
+      <c r="C8" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="D8" s="0" t="s">
+      <c r="D8" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="E8" s="0" t="s">
+      <c r="E8" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="F8" s="0" t="s">
+      <c r="F8" s="1" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
         <v>42</v>
       </c>
@@ -943,7 +949,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
         <v>50</v>
       </c>
@@ -969,227 +975,264 @@
         <v>55</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="B14" s="0" t="s">
+      <c r="B14" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="C14" s="0" t="s">
+      <c r="C14" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="D14" s="0" t="s">
+      <c r="D14" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="E14" s="0" t="s">
+      <c r="E14" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="F14" s="0" t="s">
+      <c r="F14" s="1" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="0" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="B15" s="0" t="s">
+      <c r="B15" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="C15" s="0" t="s">
+      <c r="C15" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="D15" s="0" t="s">
+      <c r="D15" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="E15" s="0" t="s">
+      <c r="E15" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="F15" s="0" t="s">
+      <c r="F15" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="H15" s="0" t="s">
+      <c r="H15" s="1" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
         <v>43</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="G19" s="6" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="H19" s="6" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="I19" s="6" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="J19" s="6" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="K19" s="6" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="L19" s="6" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="M19" s="6" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="N19" s="6" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="O19" s="6" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="P19" s="6" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B20" s="7" t="s">
         <v>32</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="E20" s="7" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F20" s="7" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="G20" s="7" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="H20" s="7" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="I20" s="7"/>
       <c r="J20" s="7" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="K20" s="7"/>
       <c r="L20" s="7"/>
       <c r="M20" s="7"/>
       <c r="N20" s="7" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="O20" s="7"/>
       <c r="P20" s="7"/>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="0" t="s">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="B21" s="0" t="s">
+      <c r="B21" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="C21" s="0" t="s">
-        <v>88</v>
-      </c>
-      <c r="D21" s="0" t="s">
+      <c r="C21" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="D21" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="E21" s="0" t="n">
+      <c r="E21" s="1" t="n">
         <v>2018</v>
       </c>
-      <c r="F21" s="0" t="n">
+      <c r="F21" s="1" t="n">
         <v>100</v>
       </c>
-      <c r="H21" s="0" t="n">
+      <c r="H21" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="I21" s="0" t="n">
+      <c r="I21" s="1" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="0" t="s">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="B22" s="0" t="s">
+      <c r="B22" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="C22" s="0" t="s">
+      <c r="C22" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="D22" s="0" t="s">
-        <v>89</v>
-      </c>
-      <c r="E22" s="0" t="n">
+      <c r="D22" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="E22" s="1" t="n">
         <v>2025</v>
       </c>
-      <c r="F22" s="0" t="n">
+      <c r="F22" s="1" t="n">
         <v>25</v>
       </c>
-      <c r="G22" s="0" t="n">
+      <c r="G22" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="H22" s="0" t="n">
+      <c r="H22" s="1" t="n">
         <v>0.65</v>
       </c>
-      <c r="I22" s="0" t="n">
+      <c r="I22" s="1" t="n">
         <v>0.74</v>
       </c>
-      <c r="J22" s="0" t="n">
+      <c r="J22" s="1" t="n">
         <f aca="false">2000/0.65/31.536</f>
         <v>97.5685907192756</v>
       </c>
-      <c r="K22" s="0" t="n">
+      <c r="K22" s="1" t="n">
         <f aca="false">1500/0.67/31.536</f>
         <v>70.9920716054431</v>
       </c>
-      <c r="L22" s="0" t="n">
+      <c r="L22" s="1" t="n">
         <f aca="false">1000/0.71/31.536</f>
         <v>44.6616788503727</v>
       </c>
-      <c r="M22" s="0" t="n">
+      <c r="M22" s="1" t="n">
         <f aca="false">750/0.74/31.536</f>
         <v>32.1383026862479</v>
       </c>
-      <c r="N22" s="0" t="n">
+      <c r="N22" s="1" t="n">
         <f aca="false">J22*0.03</f>
         <v>2.92705772157827</v>
       </c>
-      <c r="O22" s="0" t="n">
+      <c r="O22" s="1" t="n">
         <f aca="false">M22*0.03</f>
         <v>0.964149080587437</v>
       </c>
-      <c r="P22" s="0" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P22" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="E23" s="1" t="n">
+        <v>2018</v>
+      </c>
+      <c r="F23" s="1" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="8" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
   </sheetData>

</xml_diff>